<commit_message>
Implemented calc. of supply chain emissions for crop production inputs and updated get_GHG
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\prod_parameters\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>f_input</t>
   </si>
@@ -119,10 +119,10 @@
     <t>m3/kWh</t>
   </si>
   <si>
-    <t>f_ecoinvent_activity</t>
-  </si>
-  <si>
-    <t>f_ecoinvent_geography</t>
+    <t>kWh/kWh</t>
+  </si>
+  <si>
+    <t>Assumes 4.95 kWh/kg (https://en.wikipedia.org/wiki/Pellet_fuel) and 1.1 kg/kg DM (ecoinvent)</t>
   </si>
 </sst>
 </file>
@@ -130,9 +130,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -143,6 +143,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -175,13 +182,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,21 +471,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5703125" customWidth="1"/>
-    <col min="8" max="8" width="34.5703125" customWidth="1"/>
-    <col min="9" max="9" width="31.7109375" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5703125" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" customWidth="1"/>
+    <col min="7" max="7" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -484,28 +491,22 @@
         <v>5</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
@@ -515,204 +516,195 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
       <c r="B3">
         <v>368</v>
       </c>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3" t="s">
+      <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="4">
+      <c r="D3" s="4">
         <f>1/11.9</f>
         <v>8.4033613445378144E-2</v>
       </c>
-      <c r="G3" t="s">
+      <c r="E3" t="s">
         <v>27</v>
       </c>
-      <c r="H3" t="s">
+      <c r="F3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="I3"/>
-    </row>
-    <row r="4" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G3"/>
+    </row>
+    <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
-      <c r="D4"/>
+      <c r="D4" s="4"/>
       <c r="E4"/>
-      <c r="F4" s="4"/>
+      <c r="F4" s="6"/>
       <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-    </row>
-    <row r="5" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>17</v>
       </c>
       <c r="B5">
         <v>4575</v>
       </c>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5" t="s">
+      <c r="C5" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="4">
+      <c r="D5" s="4">
         <f>1/11.8</f>
         <v>8.4745762711864403E-2</v>
       </c>
-      <c r="G5" t="s">
+      <c r="E5" t="s">
         <v>27</v>
       </c>
-      <c r="H5" t="s">
+      <c r="F5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I5"/>
-    </row>
-    <row r="6" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G5"/>
+    </row>
+    <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>18</v>
       </c>
       <c r="B6">
         <v>482</v>
       </c>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6" t="s">
+      <c r="C6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="4">
+      <c r="D6" s="4">
         <f>1/10</f>
         <v>0.1</v>
       </c>
-      <c r="G6" t="s">
+      <c r="E6" t="s">
         <v>30</v>
       </c>
-      <c r="H6" t="s">
+      <c r="F6" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I6"/>
-    </row>
-    <row r="7" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G6"/>
+    </row>
+    <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
-      <c r="D7"/>
+      <c r="D7" s="4"/>
       <c r="E7"/>
-      <c r="F7" s="4"/>
+      <c r="F7" s="6"/>
       <c r="G7"/>
-      <c r="H7"/>
-      <c r="I7"/>
-    </row>
-    <row r="8" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
-      <c r="D8"/>
+      <c r="D8" s="4"/>
       <c r="E8"/>
-      <c r="F8" s="4"/>
+      <c r="F8" s="6"/>
       <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8"/>
-    </row>
-    <row r="9" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9" s="4"/>
+      <c r="B9">
+        <v>8241</v>
+      </c>
+      <c r="C9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="6"/>
       <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9"/>
-    </row>
-    <row r="10" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10"/>
+      <c r="D10" s="4"/>
       <c r="E10"/>
-      <c r="F10" s="4"/>
+      <c r="F10" s="6"/>
       <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
-    </row>
-    <row r="11" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>22</v>
       </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" s="4"/>
       <c r="E11"/>
-      <c r="F11" s="4"/>
+      <c r="F11" s="6"/>
       <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11"/>
-    </row>
-    <row r="12" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12"/>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" s="4"/>
       <c r="E12"/>
-      <c r="F12" s="4"/>
+      <c r="F12" s="6"/>
       <c r="G12"/>
-      <c r="H12"/>
-      <c r="I12"/>
-    </row>
-    <row r="13" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>23</v>
       </c>
-      <c r="B13"/>
-      <c r="C13"/>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13" s="4"/>
+      <c r="B13">
+        <v>5318</v>
+      </c>
+      <c r="C13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="4">
+        <f>1.1/4.95</f>
+        <v>0.22222222222222224</v>
+      </c>
+      <c r="E13" t="s">
+        <v>27</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>32</v>
+      </c>
       <c r="G13"/>
-      <c r="H13"/>
-      <c r="I13"/>
-    </row>
-    <row r="14" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
       <c r="B14"/>
       <c r="C14"/>
-      <c r="D14"/>
+      <c r="D14" s="4"/>
       <c r="E14"/>
-      <c r="F14" s="4"/>
+      <c r="F14" s="6"/>
       <c r="G14"/>
-      <c r="H14"/>
-      <c r="I14"/>
-    </row>
-    <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15"/>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" s="4"/>
       <c r="E15"/>
-      <c r="F15" s="4"/>
+      <c r="F15" s="6"/>
       <c r="G15"/>
-      <c r="H15"/>
-      <c r="I15"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>2</v>
       </c>
@@ -720,78 +712,77 @@
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
+      <c r="F16" s="7"/>
       <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>1</v>
       </c>
       <c r="B17">
         <v>23770</v>
       </c>
-      <c r="E17" t="s">
+      <c r="C17" t="s">
         <v>25</v>
       </c>
-      <c r="F17" s="4">
+      <c r="D17" s="4">
         <f>1/0.35</f>
         <v>2.8571428571428572</v>
       </c>
-      <c r="G17" t="s">
+      <c r="E17" t="s">
         <v>11</v>
       </c>
-      <c r="H17" t="s">
+      <c r="F17" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>3</v>
       </c>
       <c r="B18">
         <v>23770</v>
       </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="4">
+        <f t="shared" ref="D18:D19" si="0">1/0.35</f>
+        <v>2.8571428571428572</v>
+      </c>
       <c r="E18" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" s="4">
-        <f t="shared" ref="F18:F19" si="0">1/0.35</f>
-        <v>2.8571428571428572</v>
-      </c>
-      <c r="G18" t="s">
         <v>11</v>
       </c>
-      <c r="H18" t="s">
+      <c r="F18" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>4</v>
       </c>
       <c r="B19">
         <v>23770</v>
       </c>
-      <c r="E19" t="s">
+      <c r="C19" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="4">
+      <c r="D19" s="4">
         <f t="shared" si="0"/>
         <v>2.8571428571428572</v>
       </c>
-      <c r="G19" t="s">
+      <c r="E19" t="s">
         <v>11</v>
       </c>
-      <c r="H19" t="s">
+      <c r="F19" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D20" s="4"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>13</v>
       </c>
@@ -799,18 +790,18 @@
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+      <c r="F21" s="7"/>
       <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F22" s="4"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F23" s="4"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D22" s="4"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D23" s="4"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -818,37 +809,35 @@
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+      <c r="F24" s="7"/>
       <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F25" s="4"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F26" s="4"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F27" s="4"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F28" s="4"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F29" s="4"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F31" s="4"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="F32" s="4"/>
-    </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F33" s="4"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D25" s="4"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D26" s="4"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D27" s="4"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D28" s="4"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D29" s="4"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D30" s="4"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D31" s="4"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D32" s="4"/>
+    </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D33" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Implemented calculations of P and K for manure + spreading + mineral fertiliser + supply chain emissions
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="38">
   <si>
     <t>f_input</t>
   </si>
@@ -38,9 +38,6 @@
     <t>Calcium ammonium nitrate</t>
   </si>
   <si>
-    <t>NPK mixtures</t>
-  </si>
-  <si>
     <t>f_ecoinvent_id</t>
   </si>
   <si>
@@ -129,6 +126,18 @@
   </si>
   <si>
     <t>is "wood chips" good here?</t>
+  </si>
+  <si>
+    <t>Compound fertiliser-N</t>
+  </si>
+  <si>
+    <t>Compound fertiliser-P</t>
+  </si>
+  <si>
+    <t>kg/kg P</t>
+  </si>
+  <si>
+    <t>1 kg P2O5 = 0.436 kg of Phosphorous as P</t>
   </si>
 </sst>
 </file>
@@ -485,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -502,27 +511,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -533,29 +542,29 @@
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>368</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D3" s="4">
         <f>1/11.9</f>
         <v>8.4033613445378144E-2</v>
       </c>
       <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>28</v>
       </c>
       <c r="G3"/>
     </row>
     <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -566,51 +575,51 @@
     </row>
     <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>4575</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D5" s="4">
         <f>1/11.8</f>
         <v>8.4745762711864403E-2</v>
       </c>
       <c r="E5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G5"/>
     </row>
     <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6">
         <v>482</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D6" s="4">
         <f>1/10</f>
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6"/>
     </row>
     <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
@@ -630,48 +639,48 @@
     </row>
     <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9">
         <v>8241</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D9" s="4">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9"/>
     </row>
     <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10">
         <v>306</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="4">
         <f>3.6</f>
         <v>3.6</v>
       </c>
       <c r="E10" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="G10"/>
     </row>
     <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11"/>
       <c r="C11"/>
@@ -691,23 +700,23 @@
     </row>
     <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13">
         <v>5318</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D13" s="4">
         <f>1.1/4.95</f>
         <v>0.22222222222222224</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G13"/>
     </row>
@@ -740,7 +749,7 @@
       <c r="F16" s="7"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -748,20 +757,20 @@
         <v>23770</v>
       </c>
       <c r="C17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D17" s="4">
         <f>1/0.35</f>
         <v>2.8571428571428572</v>
       </c>
       <c r="E17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -769,47 +778,47 @@
         <v>23770</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D18" s="4">
         <f t="shared" ref="D18:D19" si="0">1/0.35</f>
         <v>2.8571428571428572</v>
       </c>
       <c r="E18" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="B19">
         <v>23770</v>
       </c>
       <c r="C19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D19" s="4">
         <f t="shared" si="0"/>
         <v>2.8571428571428572</v>
       </c>
       <c r="E19" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D20" s="4"/>
       <c r="F20" s="6"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -818,17 +827,35 @@
       <c r="F21" s="7"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D22" s="4"/>
-      <c r="F22" s="6"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22">
+        <v>23127</v>
+      </c>
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="4">
+        <f>1/0.436</f>
+        <v>2.2935779816513762</v>
+      </c>
+      <c r="E22" t="s">
+        <v>36</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D23" s="4"/>
       <c r="F23" s="6"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="L23" s="4"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -837,28 +864,28 @@
       <c r="F24" s="7"/>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D25" s="4"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D26" s="4"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D27" s="4"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D28" s="4"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D29" s="4"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D30" s="4"/>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D31" s="4"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D32" s="4"/>
     </row>
     <row r="33" spans="4:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Parameters for K requirements + N and P for more crops
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
   <si>
     <t>f_input</t>
   </si>
@@ -32,9 +32,6 @@
     <t>Ammonium nitrate</t>
   </si>
   <si>
-    <t>N fertilisers</t>
-  </si>
-  <si>
     <t>Calcium ammonium nitrate</t>
   </si>
   <si>
@@ -62,12 +59,6 @@
     <t>Energy</t>
   </si>
   <si>
-    <t>P fertilisers</t>
-  </si>
-  <si>
-    <t>K fertilisers</t>
-  </si>
-  <si>
     <t>Diesel</t>
   </si>
   <si>
@@ -95,9 +86,6 @@
     <t>Woody biofuels</t>
   </si>
   <si>
-    <t>1 kg ammonium nitrate = 0.35 kg of Nitrogen as N</t>
-  </si>
-  <si>
     <t>input_to_ecoinvent</t>
   </si>
   <si>
@@ -138,14 +126,24 @@
   </si>
   <si>
     <t>1 kg P2O5 = 0.436 kg of Phosphorous as P</t>
+  </si>
+  <si>
+    <t>Fertilisers</t>
+  </si>
+  <si>
+    <t>Compound fertiliser-K</t>
+  </si>
+  <si>
+    <t>1 kg K2O = 0.436 kg of Phosphorous as P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -204,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -214,6 +212,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,7 +493,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -511,27 +510,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -542,29 +541,29 @@
     </row>
     <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>368</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D3" s="4">
         <f>1/11.9</f>
         <v>8.4033613445378144E-2</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G3"/>
     </row>
     <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -575,51 +574,51 @@
     </row>
     <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>4575</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" s="4">
         <f>1/11.8</f>
         <v>8.4745762711864403E-2</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="G5"/>
     </row>
     <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>482</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4">
         <f>1/10</f>
         <v>0.1</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="G6"/>
     </row>
     <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B7"/>
       <c r="C7"/>
@@ -639,48 +638,48 @@
     </row>
     <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B9">
         <v>8241</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D9" s="4">
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9"/>
     </row>
     <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B10">
         <v>306</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4">
         <f>3.6</f>
         <v>3.6</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="G10"/>
     </row>
     <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B11"/>
       <c r="C11"/>
@@ -700,23 +699,23 @@
     </row>
     <row r="13" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B13">
         <v>5318</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D13" s="4">
         <f>1.1/4.95</f>
         <v>0.22222222222222224</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G13"/>
     </row>
@@ -740,7 +739,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -754,115 +753,108 @@
         <v>1</v>
       </c>
       <c r="B17">
-        <v>23770</v>
+        <v>23100</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="4">
-        <f>1/0.35</f>
-        <v>2.8571428571428572</v>
+        <v>20</v>
+      </c>
+      <c r="D17" s="9">
+        <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>23</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18">
-        <v>23770</v>
+        <v>23100</v>
       </c>
       <c r="C18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="4">
-        <f t="shared" ref="D18:D19" si="0">1/0.35</f>
-        <v>2.8571428571428572</v>
+        <v>20</v>
+      </c>
+      <c r="D18" s="9">
+        <v>1</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>23</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B19">
-        <v>23770</v>
+        <v>23100</v>
       </c>
       <c r="C19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="4">
-        <f t="shared" si="0"/>
-        <v>2.8571428571428572</v>
+        <v>20</v>
+      </c>
+      <c r="D19" s="9">
+        <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>23</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D20" s="4"/>
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22">
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21">
         <v>23127</v>
       </c>
-      <c r="C22" t="s">
-        <v>24</v>
-      </c>
-      <c r="D22" s="4">
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="4">
         <f>1/0.436</f>
         <v>2.2935779816513762</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E21" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D22" s="4"/>
+      <c r="F22" s="6"/>
+      <c r="L22" s="4"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23">
+        <v>22724</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="4">
+        <f>1/0.8301</f>
+        <v>1.2046741356463078</v>
+      </c>
+      <c r="E23" t="s">
+        <v>32</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F22" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D23" s="4"/>
-      <c r="F23" s="6"/>
-      <c r="L23" s="4"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="1"/>
+      <c r="D24" s="4"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D25" s="4"/>
@@ -884,12 +876,6 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D33" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added calc. of lime emissions and supply chain emissions + data
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="53">
   <si>
     <t>f_input</t>
   </si>
@@ -128,9 +128,6 @@
     <t>1 kg P2O5 = 0.436 kg of Phosphorous as P</t>
   </si>
   <si>
-    <t>Fertilisers</t>
-  </si>
-  <si>
     <t>Compound fertiliser-K</t>
   </si>
   <si>
@@ -174,6 +171,18 @@
   </si>
   <si>
     <t>Tobias Gustavsson Binder (2024) HVO100 i ljuset av Sveriges och EU:s nya klimatpolitik. IVL. https://diva-portal.org/smash/record.jsf?pid=diva2%3A1859985</t>
+  </si>
+  <si>
+    <t>Fertilisers and lime</t>
+  </si>
+  <si>
+    <t>Limestone</t>
+  </si>
+  <si>
+    <t>Dolmite</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/18042/documentation</t>
   </si>
 </sst>
 </file>
@@ -184,7 +193,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -237,6 +246,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -273,10 +290,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -295,8 +313,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -575,7 +595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M110"/>
+  <dimension ref="A1:M113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -596,7 +616,7 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>4</v>
@@ -616,7 +636,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -831,7 +851,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -927,7 +947,7 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B22">
         <v>22724</v>
@@ -943,105 +963,75 @@
         <v>32</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E23" s="4"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="13"/>
-      <c r="H24" s="13"/>
+      <c r="A24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24">
+        <v>14865</v>
+      </c>
+      <c r="D24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E24" s="4">
+        <v>1</v>
+      </c>
+      <c r="G24" s="6"/>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="14"/>
+      <c r="A25" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25">
+        <v>18042</v>
+      </c>
+      <c r="D25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="4">
+        <v>1</v>
+      </c>
+      <c r="G25" s="6"/>
+      <c r="H25" s="18" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="E26" s="14"/>
+      <c r="E26" s="4"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E27" s="14"/>
-    </row>
-    <row r="28" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28"/>
-      <c r="C28" t="s">
+      <c r="A27" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="D28" t="s">
-        <v>39</v>
-      </c>
-      <c r="E28" s="16">
-        <f>(10.5/1000)/(1/3.6)</f>
-        <v>3.78E-2</v>
-      </c>
-      <c r="F28" t="s">
-        <v>22</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H28" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>12</v>
-      </c>
-      <c r="B29"/>
-      <c r="C29" t="s">
-        <v>45</v>
-      </c>
-      <c r="D29" t="s">
-        <v>39</v>
-      </c>
-      <c r="E29" s="17">
-        <v>0</v>
-      </c>
-      <c r="F29" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="H29"/>
-    </row>
-    <row r="30" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>12</v>
-      </c>
-      <c r="B30"/>
-      <c r="C30" t="s">
+      <c r="E28" s="14"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D30" t="s">
-        <v>39</v>
-      </c>
-      <c r="E30" s="17">
-        <v>0</v>
-      </c>
-      <c r="F30" t="s">
-        <v>22</v>
-      </c>
-      <c r="G30" s="6"/>
-      <c r="H30"/>
+      <c r="E29" s="14"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
@@ -1049,40 +1039,57 @@
       </c>
       <c r="B31"/>
       <c r="C31" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D31" t="s">
-        <v>39</v>
-      </c>
-      <c r="E31" s="17">
-        <v>0</v>
+        <v>38</v>
+      </c>
+      <c r="E31" s="16">
+        <f>(10.5/1000)/(1/3.6)</f>
+        <v>3.78E-2</v>
       </c>
       <c r="F31" t="s">
         <v>22</v>
       </c>
-      <c r="G31" s="6"/>
-      <c r="H31"/>
+      <c r="G31" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H31" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="32" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32"/>
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
       <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32" s="16"/>
-      <c r="F32"/>
-      <c r="G32" s="6"/>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" s="17">
+        <v>0</v>
+      </c>
+      <c r="F32" t="s">
+        <v>22</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>47</v>
+      </c>
       <c r="H32"/>
     </row>
     <row r="33" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B33"/>
       <c r="C33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E33" s="17">
         <v>0</v>
@@ -1093,15 +1100,16 @@
       <c r="G33" s="6"/>
       <c r="H33"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>18</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B34"/>
       <c r="C34" t="s">
         <v>45</v>
       </c>
       <c r="D34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E34" s="17">
         <v>0</v>
@@ -1109,33 +1117,29 @@
       <c r="F34" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" t="s">
-        <v>43</v>
-      </c>
-      <c r="D35" t="s">
-        <v>39</v>
-      </c>
-      <c r="E35" s="17">
-        <v>0</v>
-      </c>
-      <c r="F35" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G34" s="6"/>
+      <c r="H34"/>
+    </row>
+    <row r="35" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35"/>
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35" s="16"/>
+      <c r="F35"/>
+      <c r="G35" s="6"/>
+      <c r="H35"/>
+    </row>
+    <row r="36" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>18</v>
       </c>
+      <c r="B36"/>
       <c r="C36" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E36" s="17">
         <v>0</v>
@@ -1143,15 +1147,59 @@
       <c r="F36" t="s">
         <v>22</v>
       </c>
+      <c r="G36" s="6"/>
+      <c r="H36"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E37" s="14"/>
+      <c r="A37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" s="17">
+        <v>0</v>
+      </c>
+      <c r="F37" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E38" s="14"/>
+      <c r="A38" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" s="17">
+        <v>0</v>
+      </c>
+      <c r="F38" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E39" s="14"/>
+      <c r="A39" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
+        <v>45</v>
+      </c>
+      <c r="D39" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="17">
+        <v>0</v>
+      </c>
+      <c r="F39" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E40" s="14"/>
@@ -1366,8 +1414,20 @@
     <row r="110" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E110" s="14"/>
     </row>
+    <row r="111" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E111" s="14"/>
+    </row>
+    <row r="112" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E112" s="14"/>
+    </row>
+    <row r="113" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E113" s="14"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H25" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added mineral P/K for organic and adjusted N_resid_crop for 'Green manure'
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="61">
   <si>
     <t>f_input</t>
   </si>
@@ -179,10 +179,34 @@
     <t>Limestone</t>
   </si>
   <si>
-    <t>Dolmite</t>
-  </si>
-  <si>
     <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/18042/documentation</t>
+  </si>
+  <si>
+    <t>Phosphate rock</t>
+  </si>
+  <si>
+    <t>Potassium sulfate</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/23293/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/14865/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/22724/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/23127/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/23538/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/23100/documentation</t>
+  </si>
+  <si>
+    <t>Dolomite</t>
   </si>
 </sst>
 </file>
@@ -595,7 +619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M113"/>
+  <dimension ref="A1:M115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -878,6 +902,9 @@
         <v>9</v>
       </c>
       <c r="G16" s="6"/>
+      <c r="H16" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -896,6 +923,9 @@
         <v>9</v>
       </c>
       <c r="G17" s="6"/>
+      <c r="H17" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -914,6 +944,9 @@
         <v>9</v>
       </c>
       <c r="G18" s="6"/>
+      <c r="H18" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E19" s="4"/>
@@ -921,10 +954,10 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="B20">
-        <v>23127</v>
+        <v>23538</v>
       </c>
       <c r="D20" t="s">
         <v>20</v>
@@ -939,146 +972,157 @@
       <c r="G20" s="6" t="s">
         <v>33</v>
       </c>
+      <c r="H20" s="18" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E21" s="4"/>
-      <c r="G21" s="6"/>
-      <c r="M21" s="4"/>
+      <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21">
+        <v>23127</v>
+      </c>
+      <c r="D21" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="4">
+        <f>1/0.436</f>
+        <v>2.2935779816513762</v>
+      </c>
+      <c r="F21" t="s">
+        <v>32</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H21" s="18" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22">
-        <v>22724</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="E22" s="4"/>
+      <c r="G22" s="6"/>
+      <c r="M22" s="4"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23">
+        <v>23293</v>
+      </c>
+      <c r="D23" t="s">
         <v>20</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E23" s="4">
         <f>1/0.8301</f>
         <v>1.2046741356463078</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F23" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G23" s="6" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E23" s="4"/>
-      <c r="G23" s="6"/>
+      <c r="H23" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="4"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B24">
-        <v>14865</v>
+        <v>22724</v>
       </c>
       <c r="D24" t="s">
         <v>20</v>
       </c>
       <c r="E24" s="4">
+        <f>1/0.8301</f>
+        <v>1.2046741356463078</v>
+      </c>
+      <c r="F24" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E25" s="4"/>
+      <c r="G25" s="6"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26">
+        <v>14865</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" s="4">
         <v>1</v>
       </c>
-      <c r="G24" s="6"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="G26" s="6"/>
+      <c r="H26" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27">
+        <v>18042</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="4">
+        <v>1</v>
+      </c>
+      <c r="G27" s="6"/>
+      <c r="H27" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B25">
-        <v>18042</v>
-      </c>
-      <c r="D25" t="s">
-        <v>20</v>
-      </c>
-      <c r="E25" s="4">
-        <v>1</v>
-      </c>
-      <c r="G25" s="6"/>
-      <c r="H25" s="18" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E26" s="4"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E28" s="14"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="E30" s="14"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E29" s="14"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E30" s="14"/>
-    </row>
-    <row r="31" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>12</v>
-      </c>
-      <c r="B31"/>
-      <c r="C31" t="s">
-        <v>40</v>
-      </c>
-      <c r="D31" t="s">
-        <v>38</v>
-      </c>
-      <c r="E31" s="16">
-        <f>(10.5/1000)/(1/3.6)</f>
-        <v>3.78E-2</v>
-      </c>
-      <c r="F31" t="s">
-        <v>22</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="H31" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32"/>
-      <c r="C32" t="s">
-        <v>44</v>
-      </c>
-      <c r="D32" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32" s="17">
-        <v>0</v>
-      </c>
-      <c r="F32" t="s">
-        <v>22</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H32"/>
+      <c r="E31" s="14"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E32" s="14"/>
     </row>
     <row r="33" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
@@ -1086,19 +1130,24 @@
       </c>
       <c r="B33"/>
       <c r="C33" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D33" t="s">
         <v>38</v>
       </c>
-      <c r="E33" s="17">
-        <v>0</v>
+      <c r="E33" s="16">
+        <f>(10.5/1000)/(1/3.6)</f>
+        <v>3.78E-2</v>
       </c>
       <c r="F33" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="6"/>
-      <c r="H33"/>
+      <c r="G33" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="H33" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="34" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -1106,7 +1155,7 @@
       </c>
       <c r="B34"/>
       <c r="C34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D34" t="s">
         <v>38</v>
@@ -1117,26 +1166,38 @@
       <c r="F34" t="s">
         <v>22</v>
       </c>
-      <c r="G34" s="6"/>
+      <c r="G34" s="8" t="s">
+        <v>47</v>
+      </c>
       <c r="H34"/>
     </row>
     <row r="35" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35"/>
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
       <c r="B35"/>
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35" s="16"/>
-      <c r="F35"/>
+      <c r="C35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D35" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="17">
+        <v>0</v>
+      </c>
+      <c r="F35" t="s">
+        <v>22</v>
+      </c>
       <c r="G35" s="6"/>
       <c r="H35"/>
     </row>
     <row r="36" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B36"/>
       <c r="C36" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D36" t="s">
         <v>38</v>
@@ -1150,29 +1211,23 @@
       <c r="G36" s="6"/>
       <c r="H36"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>18</v>
-      </c>
-      <c r="C37" t="s">
-        <v>44</v>
-      </c>
-      <c r="D37" t="s">
-        <v>38</v>
-      </c>
-      <c r="E37" s="17">
-        <v>0</v>
-      </c>
-      <c r="F37" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37" s="16"/>
+      <c r="F37"/>
+      <c r="G37" s="6"/>
+      <c r="H37"/>
+    </row>
+    <row r="38" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>18</v>
       </c>
+      <c r="B38"/>
       <c r="C38" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D38" t="s">
         <v>38</v>
@@ -1183,13 +1238,15 @@
       <c r="F38" t="s">
         <v>22</v>
       </c>
+      <c r="G38" s="6"/>
+      <c r="H38"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>18</v>
       </c>
       <c r="C39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D39" t="s">
         <v>38</v>
@@ -1202,10 +1259,38 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E40" s="14"/>
+      <c r="A40" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="17">
+        <v>0</v>
+      </c>
+      <c r="F40" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E41" s="14"/>
+      <c r="A41" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" t="s">
+        <v>45</v>
+      </c>
+      <c r="D41" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="17">
+        <v>0</v>
+      </c>
+      <c r="F41" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E42" s="14"/>
@@ -1423,11 +1508,25 @@
     <row r="113" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E113" s="14"/>
     </row>
+    <row r="114" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E114" s="14"/>
+    </row>
+    <row r="115" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E115" s="14"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H25" r:id="rId1"/>
+    <hyperlink ref="H27" r:id="rId1"/>
+    <hyperlink ref="H23" r:id="rId2"/>
+    <hyperlink ref="H26" r:id="rId3"/>
+    <hyperlink ref="H24" r:id="rId4"/>
+    <hyperlink ref="H21" r:id="rId5"/>
+    <hyperlink ref="H20" r:id="rId6"/>
+    <hyperlink ref="H18" r:id="rId7"/>
+    <hyperlink ref="H17" r:id="rId8"/>
+    <hyperlink ref="H16" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added some non-GHG compounds to InputsMgmt and combustion emissions
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F74B10A-C80E-455E-8220-8A5F93B2B485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6900"/>
+    <workbookView xWindow="-25320" yWindow="2055" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
   <si>
     <t>f_input</t>
   </si>
@@ -125,15 +137,9 @@
     <t>kg/kg P</t>
   </si>
   <si>
-    <t>1 kg P2O5 = 0.436 kg of Phosphorous as P</t>
-  </si>
-  <si>
     <t>Compound fertiliser-K</t>
   </si>
   <si>
-    <t>1 kg K2O = 0.436 kg of Phosphorous as P</t>
-  </si>
-  <si>
     <t>Ecoinvent connections</t>
   </si>
   <si>
@@ -207,12 +213,39 @@
   </si>
   <si>
     <t>Dolomite</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/368/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/4575/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/482/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/8241/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/306/documentation</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.10/cutoff/dataset/5318/documentation</t>
+  </si>
+  <si>
+    <t>kg/kg K</t>
+  </si>
+  <si>
+    <t>1 kg K2O = 0.8301 kg K</t>
+  </si>
+  <si>
+    <t>1 kg P2O5 = 0.436 kg P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
@@ -318,13 +351,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -618,7 +650,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M115"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -640,7 +672,7 @@
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>4</v>
@@ -659,16 +691,16 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="A2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -682,14 +714,13 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
       <c r="B4">
         <v>368</v>
       </c>
-      <c r="C4"/>
       <c r="D4" t="s">
         <v>20</v>
       </c>
@@ -700,31 +731,27 @@
       <c r="F4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H4"/>
-    </row>
-    <row r="5" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H4" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
       <c r="E5" s="4"/>
-      <c r="F5"/>
-      <c r="G5" s="6"/>
-      <c r="H5"/>
-    </row>
-    <row r="6" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6">
         <v>4575</v>
       </c>
-      <c r="C6"/>
       <c r="D6" t="s">
         <v>20</v>
       </c>
@@ -735,19 +762,20 @@
       <c r="F6" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H6"/>
-    </row>
-    <row r="7" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H6" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="B7">
         <v>482</v>
       </c>
-      <c r="C7"/>
       <c r="D7" t="s">
         <v>20</v>
       </c>
@@ -758,41 +786,31 @@
       <c r="F7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="H7"/>
-    </row>
-    <row r="8" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H7" s="17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
       <c r="E8" s="4"/>
-      <c r="F8"/>
-      <c r="G8" s="6"/>
-      <c r="H8"/>
-    </row>
-    <row r="9" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9"/>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
+      <c r="G8" s="5"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E9" s="4"/>
-      <c r="F9"/>
-      <c r="G9" s="6"/>
-      <c r="H9"/>
-    </row>
-    <row r="10" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
       <c r="B10">
         <v>8241</v>
       </c>
-      <c r="C10"/>
       <c r="D10" t="s">
         <v>20</v>
       </c>
@@ -802,17 +820,18 @@
       <c r="F10" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="6"/>
-      <c r="H10"/>
-    </row>
-    <row r="11" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G10" s="5"/>
+      <c r="H10" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11">
         <v>306</v>
       </c>
-      <c r="C11"/>
       <c r="D11" t="s">
         <v>20</v>
       </c>
@@ -823,31 +842,27 @@
       <c r="F11" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="G11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H11"/>
-    </row>
-    <row r="12" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="H11" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12"/>
-      <c r="C12"/>
-      <c r="D12"/>
       <c r="E12" s="4"/>
-      <c r="F12"/>
-      <c r="G12" s="6"/>
-      <c r="H12"/>
-    </row>
-    <row r="13" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G12" s="5"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
       <c r="B13">
         <v>5318</v>
       </c>
-      <c r="C13"/>
       <c r="D13" t="s">
         <v>20</v>
       </c>
@@ -858,31 +873,27 @@
       <c r="F13" t="s">
         <v>22</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H13"/>
-    </row>
-    <row r="14" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14"/>
-      <c r="B14"/>
-      <c r="C14"/>
-      <c r="D14"/>
+      <c r="H13" s="17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E14" s="4"/>
-      <c r="F14"/>
-      <c r="G14" s="6"/>
-      <c r="H14"/>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="7"/>
+      <c r="G15" s="6"/>
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -895,15 +906,15 @@
       <c r="D16" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="9">
+      <c r="E16" s="8">
         <v>1</v>
       </c>
       <c r="F16" t="s">
         <v>9</v>
       </c>
-      <c r="G16" s="6"/>
-      <c r="H16" s="18" t="s">
-        <v>59</v>
+      <c r="G16" s="5"/>
+      <c r="H16" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
@@ -916,15 +927,15 @@
       <c r="D17" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="9">
+      <c r="E17" s="8">
         <v>1</v>
       </c>
       <c r="F17" t="s">
         <v>9</v>
       </c>
-      <c r="G17" s="6"/>
-      <c r="H17" s="18" t="s">
-        <v>59</v>
+      <c r="G17" s="5"/>
+      <c r="H17" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
@@ -937,24 +948,24 @@
       <c r="D18" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="8">
         <v>1</v>
       </c>
       <c r="F18" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="6"/>
-      <c r="H18" s="18" t="s">
-        <v>59</v>
+      <c r="G18" s="5"/>
+      <c r="H18" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E19" s="4"/>
-      <c r="G19" s="6"/>
+      <c r="G19" s="5"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20">
         <v>23538</v>
@@ -969,11 +980,11 @@
       <c r="F20" t="s">
         <v>32</v>
       </c>
-      <c r="G20" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H20" s="18" t="s">
-        <v>58</v>
+      <c r="G20" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="17" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
@@ -993,21 +1004,21 @@
       <c r="F21" t="s">
         <v>32</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H21" s="18" t="s">
-        <v>57</v>
+      <c r="G21" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E22" s="4"/>
-      <c r="G22" s="6"/>
+      <c r="G22" s="5"/>
       <c r="M22" s="4"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B23">
         <v>23293</v>
@@ -1020,19 +1031,19 @@
         <v>1.2046741356463078</v>
       </c>
       <c r="F23" t="s">
-        <v>32</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" s="18" t="s">
-        <v>54</v>
+        <v>65</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>52</v>
       </c>
       <c r="M23" s="4"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24">
         <v>22724</v>
@@ -1045,22 +1056,22 @@
         <v>1.2046741356463078</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H24" s="18" t="s">
-        <v>56</v>
+        <v>65</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E25" s="4"/>
-      <c r="G25" s="6"/>
+      <c r="G25" s="5"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B26">
         <v>14865</v>
@@ -1071,14 +1082,14 @@
       <c r="E26" s="4">
         <v>1</v>
       </c>
-      <c r="G26" s="6"/>
-      <c r="H26" s="18" t="s">
-        <v>55</v>
+      <c r="G26" s="5"/>
+      <c r="H26" s="17" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B27">
         <v>18042</v>
@@ -1089,169 +1100,154 @@
       <c r="E27" s="4">
         <v>1</v>
       </c>
-      <c r="G27" s="6"/>
-      <c r="H27" s="18" t="s">
-        <v>51</v>
+      <c r="G27" s="5"/>
+      <c r="H27" s="17" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E28" s="4"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
+      <c r="A29" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="13"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E30" s="14"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="E31" s="14"/>
+      <c r="E31" s="13"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E32" s="14"/>
-    </row>
-    <row r="33" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="E32" s="13"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>12</v>
       </c>
-      <c r="B33"/>
       <c r="C33" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D33" t="s">
-        <v>38</v>
-      </c>
-      <c r="E33" s="16">
+        <v>36</v>
+      </c>
+      <c r="E33" s="15">
         <f>(10.5/1000)/(1/3.6)</f>
         <v>3.78E-2</v>
       </c>
       <c r="F33" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="G33" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" t="s">
         <v>46</v>
       </c>
-      <c r="H33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>12</v>
       </c>
-      <c r="B34"/>
       <c r="C34" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D34" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="17">
+        <v>36</v>
+      </c>
+      <c r="E34" s="16">
         <v>0</v>
       </c>
       <c r="F34" t="s">
         <v>22</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="H34"/>
-    </row>
-    <row r="35" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G34" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>12</v>
       </c>
-      <c r="B35"/>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D35" t="s">
-        <v>38</v>
-      </c>
-      <c r="E35" s="17">
+        <v>36</v>
+      </c>
+      <c r="E35" s="16">
         <v>0</v>
       </c>
       <c r="F35" t="s">
         <v>22</v>
       </c>
-      <c r="G35" s="6"/>
-      <c r="H35"/>
-    </row>
-    <row r="36" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G35" s="5"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>12</v>
       </c>
-      <c r="B36"/>
       <c r="C36" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D36" t="s">
-        <v>38</v>
-      </c>
-      <c r="E36" s="17">
+        <v>36</v>
+      </c>
+      <c r="E36" s="16">
         <v>0</v>
       </c>
       <c r="F36" t="s">
         <v>22</v>
       </c>
-      <c r="G36" s="6"/>
-      <c r="H36"/>
-    </row>
-    <row r="37" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37" s="16"/>
-      <c r="F37"/>
-      <c r="G37" s="6"/>
-      <c r="H37"/>
-    </row>
-    <row r="38" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E37" s="15"/>
+      <c r="G37" s="5"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>18</v>
       </c>
-      <c r="B38"/>
       <c r="C38" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
-      </c>
-      <c r="E38" s="17">
+        <v>36</v>
+      </c>
+      <c r="E38" s="16">
         <v>0</v>
       </c>
       <c r="F38" t="s">
         <v>22</v>
       </c>
-      <c r="G38" s="6"/>
-      <c r="H38"/>
+      <c r="G38" s="5"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>18</v>
       </c>
       <c r="C39" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D39" t="s">
-        <v>38</v>
-      </c>
-      <c r="E39" s="17">
+        <v>36</v>
+      </c>
+      <c r="E39" s="16">
         <v>0</v>
       </c>
       <c r="F39" t="s">
@@ -1263,12 +1259,12 @@
         <v>18</v>
       </c>
       <c r="C40" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
-      </c>
-      <c r="E40" s="17">
+        <v>36</v>
+      </c>
+      <c r="E40" s="16">
         <v>0</v>
       </c>
       <c r="F40" t="s">
@@ -1280,12 +1276,12 @@
         <v>18</v>
       </c>
       <c r="C41" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
-      </c>
-      <c r="E41" s="17">
+        <v>36</v>
+      </c>
+      <c r="E41" s="16">
         <v>0</v>
       </c>
       <c r="F41" t="s">
@@ -1293,240 +1289,246 @@
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E42" s="14"/>
+      <c r="E42" s="13"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E43" s="14"/>
+      <c r="E43" s="13"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E44" s="14"/>
+      <c r="E44" s="13"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E45" s="14"/>
+      <c r="E45" s="13"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E46" s="14"/>
+      <c r="E46" s="13"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E47" s="14"/>
+      <c r="E47" s="13"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E48" s="14"/>
+      <c r="E48" s="13"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E49" s="14"/>
+      <c r="E49" s="13"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E50" s="14"/>
+      <c r="E50" s="13"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E51" s="14"/>
+      <c r="E51" s="13"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E52" s="14"/>
+      <c r="E52" s="13"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E53" s="14"/>
+      <c r="E53" s="13"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E54" s="14"/>
+      <c r="E54" s="13"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E55" s="14"/>
+      <c r="E55" s="13"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E56" s="14"/>
+      <c r="E56" s="13"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E57" s="14"/>
+      <c r="E57" s="13"/>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E58" s="14"/>
+      <c r="E58" s="13"/>
     </row>
     <row r="59" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E59" s="14"/>
+      <c r="E59" s="13"/>
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E60" s="14"/>
+      <c r="E60" s="13"/>
     </row>
     <row r="61" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E61" s="14"/>
+      <c r="E61" s="13"/>
     </row>
     <row r="62" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E62" s="14"/>
+      <c r="E62" s="13"/>
     </row>
     <row r="63" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E63" s="14"/>
+      <c r="E63" s="13"/>
     </row>
     <row r="64" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E64" s="14"/>
+      <c r="E64" s="13"/>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E65" s="14"/>
+      <c r="E65" s="13"/>
     </row>
     <row r="66" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E66" s="14"/>
+      <c r="E66" s="13"/>
     </row>
     <row r="67" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E67" s="14"/>
+      <c r="E67" s="13"/>
     </row>
     <row r="68" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E68" s="14"/>
+      <c r="E68" s="13"/>
     </row>
     <row r="69" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E69" s="14"/>
+      <c r="E69" s="13"/>
     </row>
     <row r="70" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E70" s="14"/>
+      <c r="E70" s="13"/>
     </row>
     <row r="71" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E71" s="14"/>
+      <c r="E71" s="13"/>
     </row>
     <row r="72" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E72" s="14"/>
+      <c r="E72" s="13"/>
     </row>
     <row r="73" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E73" s="14"/>
+      <c r="E73" s="13"/>
     </row>
     <row r="74" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E74" s="14"/>
+      <c r="E74" s="13"/>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E75" s="14"/>
+      <c r="E75" s="13"/>
     </row>
     <row r="76" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E76" s="14"/>
+      <c r="E76" s="13"/>
     </row>
     <row r="77" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E77" s="14"/>
+      <c r="E77" s="13"/>
     </row>
     <row r="78" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E78" s="14"/>
+      <c r="E78" s="13"/>
     </row>
     <row r="79" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E79" s="14"/>
+      <c r="E79" s="13"/>
     </row>
     <row r="80" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E80" s="14"/>
+      <c r="E80" s="13"/>
     </row>
     <row r="81" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E81" s="14"/>
+      <c r="E81" s="13"/>
     </row>
     <row r="82" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E82" s="14"/>
+      <c r="E82" s="13"/>
     </row>
     <row r="83" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E83" s="14"/>
+      <c r="E83" s="13"/>
     </row>
     <row r="84" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E84" s="14"/>
+      <c r="E84" s="13"/>
     </row>
     <row r="85" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E85" s="14"/>
+      <c r="E85" s="13"/>
     </row>
     <row r="86" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E86" s="14"/>
+      <c r="E86" s="13"/>
     </row>
     <row r="87" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E87" s="14"/>
+      <c r="E87" s="13"/>
     </row>
     <row r="88" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E88" s="14"/>
+      <c r="E88" s="13"/>
     </row>
     <row r="89" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E89" s="14"/>
+      <c r="E89" s="13"/>
     </row>
     <row r="90" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E90" s="14"/>
+      <c r="E90" s="13"/>
     </row>
     <row r="91" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E91" s="14"/>
+      <c r="E91" s="13"/>
     </row>
     <row r="92" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E92" s="14"/>
+      <c r="E92" s="13"/>
     </row>
     <row r="93" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E93" s="14"/>
+      <c r="E93" s="13"/>
     </row>
     <row r="94" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E94" s="14"/>
+      <c r="E94" s="13"/>
     </row>
     <row r="95" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E95" s="14"/>
+      <c r="E95" s="13"/>
     </row>
     <row r="96" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E96" s="14"/>
+      <c r="E96" s="13"/>
     </row>
     <row r="97" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E97" s="14"/>
+      <c r="E97" s="13"/>
     </row>
     <row r="98" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E98" s="14"/>
+      <c r="E98" s="13"/>
     </row>
     <row r="99" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E99" s="14"/>
+      <c r="E99" s="13"/>
     </row>
     <row r="100" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E100" s="14"/>
+      <c r="E100" s="13"/>
     </row>
     <row r="101" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E101" s="14"/>
+      <c r="E101" s="13"/>
     </row>
     <row r="102" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E102" s="14"/>
+      <c r="E102" s="13"/>
     </row>
     <row r="103" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E103" s="14"/>
+      <c r="E103" s="13"/>
     </row>
     <row r="104" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E104" s="14"/>
+      <c r="E104" s="13"/>
     </row>
     <row r="105" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E105" s="14"/>
+      <c r="E105" s="13"/>
     </row>
     <row r="106" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E106" s="14"/>
+      <c r="E106" s="13"/>
     </row>
     <row r="107" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E107" s="14"/>
+      <c r="E107" s="13"/>
     </row>
     <row r="108" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E108" s="14"/>
+      <c r="E108" s="13"/>
     </row>
     <row r="109" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E109" s="14"/>
+      <c r="E109" s="13"/>
     </row>
     <row r="110" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E110" s="14"/>
+      <c r="E110" s="13"/>
     </row>
     <row r="111" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E111" s="14"/>
+      <c r="E111" s="13"/>
     </row>
     <row r="112" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E112" s="14"/>
+      <c r="E112" s="13"/>
     </row>
     <row r="113" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E113" s="14"/>
+      <c r="E113" s="13"/>
     </row>
     <row r="114" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E114" s="14"/>
+      <c r="E114" s="13"/>
     </row>
     <row r="115" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E115" s="14"/>
+      <c r="E115" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H27" r:id="rId1"/>
-    <hyperlink ref="H23" r:id="rId2"/>
-    <hyperlink ref="H26" r:id="rId3"/>
-    <hyperlink ref="H24" r:id="rId4"/>
-    <hyperlink ref="H21" r:id="rId5"/>
-    <hyperlink ref="H20" r:id="rId6"/>
-    <hyperlink ref="H18" r:id="rId7"/>
-    <hyperlink ref="H17" r:id="rId8"/>
-    <hyperlink ref="H16" r:id="rId9"/>
+    <hyperlink ref="H27" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="H23" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="H26" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="H24" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="H21" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="H20" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="H18" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="H17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="H16" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="H4" r:id="rId10" xr:uid="{685707BE-1BCE-4E9F-99EB-1613360E2FC0}"/>
+    <hyperlink ref="H6" r:id="rId11" xr:uid="{6E3BC458-1BD9-4220-A828-70E703A50CA8}"/>
+    <hyperlink ref="H7" r:id="rId12" xr:uid="{2B49D38A-28EC-4146-8000-9A604AE3B755}"/>
+    <hyperlink ref="H10" r:id="rId13" xr:uid="{30CE8B64-F407-41BB-AFA8-3DAB94354661}"/>
+    <hyperlink ref="H11" r:id="rId14" xr:uid="{DA87E9D9-5066-46DD-8FCA-E6FB6C91821A}"/>
+    <hyperlink ref="H13" r:id="rId15" xr:uid="{E9108AA1-47D0-4D91-95C1-CB5183B49E5E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Wastewater treatment energy and input use in InputsMgmt + data for NaOH as input
</commit_message>
<xml_diff>
--- a/data/default/InputsMgmt.xlsx
+++ b/data/default/InputsMgmt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F74B10A-C80E-455E-8220-8A5F93B2B485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71CBFA45-4F8E-476A-AF8D-7ADD727E8EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="2055" windowWidth="25440" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="73">
   <si>
     <t>f_input</t>
   </si>
@@ -240,6 +240,21 @@
   </si>
   <si>
     <t>1 kg P2O5 = 0.436 kg P</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Sodium hydroxide</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.12/cutoff/dataset/29617/documentation</t>
+  </si>
+  <si>
+    <t>50% NaOH solution</t>
+  </si>
+  <si>
+    <t>kg NaOH solution/kg NaOH</t>
   </si>
 </sst>
 </file>
@@ -651,7 +666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M115"/>
+  <dimension ref="A1:M119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
@@ -1107,124 +1122,109 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="E28" s="4"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="1"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B30">
+        <v>29617</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" s="8">
+        <v>2</v>
+      </c>
+      <c r="F30" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="H30" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E31" s="4"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="17"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E32" s="4"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="E30" s="13"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
+      <c r="E34" s="13"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="E31" s="13"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E32" s="13"/>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="E35" s="13"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E36" s="13"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>12</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C37" t="s">
         <v>38</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D37" t="s">
         <v>36</v>
       </c>
-      <c r="E33" s="15">
+      <c r="E37" s="15">
         <f>(10.5/1000)/(1/3.6)</f>
         <v>3.78E-2</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F37" t="s">
         <v>22</v>
       </c>
-      <c r="G33" s="5" t="s">
+      <c r="G37" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H33" t="s">
+      <c r="H37" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" t="s">
-        <v>42</v>
-      </c>
-      <c r="D34" t="s">
-        <v>36</v>
-      </c>
-      <c r="E34" s="16">
-        <v>0</v>
-      </c>
-      <c r="F34" t="s">
-        <v>22</v>
-      </c>
-      <c r="G34" s="7" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" t="s">
-        <v>36</v>
-      </c>
-      <c r="E35" s="16">
-        <v>0</v>
-      </c>
-      <c r="F35" t="s">
-        <v>22</v>
-      </c>
-      <c r="G35" s="5"/>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" t="s">
-        <v>43</v>
-      </c>
-      <c r="D36" t="s">
-        <v>36</v>
-      </c>
-      <c r="E36" s="16">
-        <v>0</v>
-      </c>
-      <c r="F36" t="s">
-        <v>22</v>
-      </c>
-      <c r="G36" s="5"/>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E37" s="15"/>
-      <c r="G37" s="5"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D38" t="s">
         <v>36</v>
@@ -1235,14 +1235,16 @@
       <c r="F38" t="s">
         <v>22</v>
       </c>
-      <c r="G38" s="5"/>
+      <c r="G38" s="7" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C39" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D39" t="s">
         <v>36</v>
@@ -1253,13 +1255,14 @@
       <c r="F39" t="s">
         <v>22</v>
       </c>
+      <c r="G39" s="5"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C40" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D40" t="s">
         <v>36</v>
@@ -1270,35 +1273,80 @@
       <c r="F40" t="s">
         <v>22</v>
       </c>
+      <c r="G40" s="5"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="E41" s="15"/>
+      <c r="G41" s="5"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>18</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C42" t="s">
+        <v>38</v>
+      </c>
+      <c r="D42" t="s">
+        <v>36</v>
+      </c>
+      <c r="E42" s="16">
+        <v>0</v>
+      </c>
+      <c r="F42" t="s">
+        <v>22</v>
+      </c>
+      <c r="G42" s="5"/>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>18</v>
+      </c>
+      <c r="C43" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" t="s">
+        <v>36</v>
+      </c>
+      <c r="E43" s="16">
+        <v>0</v>
+      </c>
+      <c r="F43" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>18</v>
+      </c>
+      <c r="C44" t="s">
+        <v>40</v>
+      </c>
+      <c r="D44" t="s">
+        <v>36</v>
+      </c>
+      <c r="E44" s="16">
+        <v>0</v>
+      </c>
+      <c r="F44" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" t="s">
         <v>43</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D45" t="s">
         <v>36</v>
       </c>
-      <c r="E41" s="16">
+      <c r="E45" s="16">
         <v>0</v>
       </c>
-      <c r="F41" t="s">
+      <c r="F45" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E42" s="13"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E43" s="13"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E44" s="13"/>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="E45" s="13"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E46" s="13"/>
@@ -1509,6 +1557,18 @@
     </row>
     <row r="115" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E115" s="13"/>
+    </row>
+    <row r="116" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E116" s="13"/>
+    </row>
+    <row r="117" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E117" s="13"/>
+    </row>
+    <row r="118" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E118" s="13"/>
+    </row>
+    <row r="119" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E119" s="13"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1527,8 +1587,9 @@
     <hyperlink ref="H10" r:id="rId13" xr:uid="{30CE8B64-F407-41BB-AFA8-3DAB94354661}"/>
     <hyperlink ref="H11" r:id="rId14" xr:uid="{DA87E9D9-5066-46DD-8FCA-E6FB6C91821A}"/>
     <hyperlink ref="H13" r:id="rId15" xr:uid="{E9108AA1-47D0-4D91-95C1-CB5183B49E5E}"/>
+    <hyperlink ref="H30" r:id="rId16" xr:uid="{9A5CB449-B215-48F5-810B-6CC7AA512DB9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId16"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId17"/>
 </worksheet>
 </file>
</xml_diff>